<commit_message>
Updated version of the AltBug Algorithm
</commit_message>
<xml_diff>
--- a/AlgorithmNData/Bug Algorithms Full Documented Values.xlsx
+++ b/AlgorithmNData/Bug Algorithms Full Documented Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utrgv-my.sharepoint.com/personal/izabella_valero01_utrgv_edu/Documents/Desktop/MARS Research/May20-PathPlanning/My_Work/Typed Reports/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utrgv-my.sharepoint.com/personal/izabella_valero01_utrgv_edu/Documents/Desktop/MARS Research/May20-PathPlanning/webots/mars-github-bug-algorithms/bug_algorithms/AlgorithmNData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1193" documentId="8_{3A44FF85-21B8-4464-9902-83D39A64E269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C34BDE7-90CE-40BA-A3C3-B189488E0301}"/>
+  <xr:revisionPtr revIDLastSave="1214" documentId="8_{3A44FF85-21B8-4464-9902-83D39A64E269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A08C817-3DB1-4618-B7F1-3433423008CB}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{1B981E3A-1744-4B50-BA68-B582BA61DD63}"/>
+    <workbookView xWindow="7973" yWindow="15" windowWidth="14527" windowHeight="11115" xr2:uid="{1B981E3A-1744-4B50-BA68-B582BA61DD63}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -513,7 +513,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -557,36 +557,11 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -612,6 +587,30 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10253,40 +10252,19 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:62" x14ac:dyDescent="0.45">
-      <c r="A3" s="37"/>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="37"/>
-      <c r="J3" s="37"/>
+      <c r="A3" s="47"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
     </row>
-    <row r="4" spans="1:62" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A4" s="38"/>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="38"/>
-      <c r="F4" s="38"/>
-      <c r="G4" s="38"/>
-      <c r="H4" s="38"/>
-      <c r="I4" s="38"/>
-      <c r="J4" s="38"/>
-    </row>
+    <row r="4" spans="1:62" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="5" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A5" s="38"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="38"/>
-      <c r="G5" s="38"/>
-      <c r="H5" s="38"/>
-      <c r="I5" s="38"/>
-      <c r="J5" s="38"/>
       <c r="O5" t="s">
         <v>42</v>
       </c>
@@ -10295,16 +10273,6 @@
       </c>
     </row>
     <row r="6" spans="1:62" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="38"/>
-      <c r="B6" s="38"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="38"/>
-      <c r="H6" s="38"/>
-      <c r="I6" s="38"/>
-      <c r="J6" s="38"/>
       <c r="N6" t="s">
         <v>35</v>
       </c>
@@ -10319,16 +10287,6 @@
       </c>
     </row>
     <row r="7" spans="1:62" x14ac:dyDescent="0.45">
-      <c r="A7" s="38"/>
-      <c r="B7" s="38"/>
-      <c r="C7" s="38"/>
-      <c r="D7" s="38"/>
-      <c r="E7" s="38"/>
-      <c r="F7" s="38"/>
-      <c r="G7" s="38"/>
-      <c r="H7" s="38"/>
-      <c r="I7" s="38"/>
-      <c r="J7" s="38"/>
       <c r="N7" t="s">
         <v>36</v>
       </c>
@@ -10343,16 +10301,6 @@
       </c>
     </row>
     <row r="8" spans="1:62" x14ac:dyDescent="0.45">
-      <c r="A8" s="38"/>
-      <c r="B8" s="38"/>
-      <c r="C8" s="38"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="38"/>
-      <c r="G8" s="38"/>
-      <c r="H8" s="38"/>
-      <c r="I8" s="38"/>
-      <c r="J8" s="38"/>
       <c r="N8" t="s">
         <v>37</v>
       </c>
@@ -10367,16 +10315,6 @@
       </c>
     </row>
     <row r="9" spans="1:62" x14ac:dyDescent="0.45">
-      <c r="A9" s="38"/>
-      <c r="B9" s="38"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="38"/>
-      <c r="H9" s="38"/>
-      <c r="I9" s="38"/>
-      <c r="J9" s="38"/>
       <c r="N9" t="s">
         <v>38</v>
       </c>
@@ -10391,16 +10329,6 @@
       </c>
     </row>
     <row r="10" spans="1:62" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A10" s="38"/>
-      <c r="B10" s="38"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="38"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="38"/>
-      <c r="G10" s="38"/>
-      <c r="H10" s="38"/>
-      <c r="I10" s="38"/>
-      <c r="J10" s="38"/>
       <c r="N10" t="s">
         <v>39</v>
       </c>
@@ -10415,16 +10343,6 @@
       </c>
     </row>
     <row r="11" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A11" s="38"/>
-      <c r="B11" s="38"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="38"/>
-      <c r="E11" s="38"/>
-      <c r="F11" s="38"/>
-      <c r="G11" s="38"/>
-      <c r="H11" s="38"/>
-      <c r="I11" s="38"/>
-      <c r="J11" s="38"/>
       <c r="N11" t="s">
         <v>40</v>
       </c>
@@ -10478,16 +10396,6 @@
       </c>
     </row>
     <row r="12" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A12" s="38"/>
-      <c r="B12" s="38"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="38"/>
-      <c r="G12" s="38"/>
-      <c r="H12" s="38"/>
-      <c r="I12" s="38"/>
-      <c r="J12" s="38"/>
       <c r="N12" t="s">
         <v>41</v>
       </c>
@@ -10544,16 +10452,13 @@
       </c>
     </row>
     <row r="13" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A13" s="37"/>
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="38"/>
-      <c r="I13" s="38"/>
-      <c r="J13" s="38"/>
+      <c r="A13" s="47"/>
+      <c r="B13" s="47"/>
+      <c r="C13" s="47"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="47"/>
+      <c r="F13" s="47"/>
+      <c r="G13" s="47"/>
       <c r="O13" s="14"/>
       <c r="AP13" t="s">
         <v>36</v>
@@ -10599,16 +10504,6 @@
       </c>
     </row>
     <row r="14" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A14" s="38"/>
-      <c r="B14" s="38"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="38"/>
-      <c r="G14" s="38"/>
-      <c r="H14" s="38"/>
-      <c r="I14" s="38"/>
-      <c r="J14" s="38"/>
       <c r="AP14" t="s">
         <v>37</v>
       </c>
@@ -10653,16 +10548,6 @@
       </c>
     </row>
     <row r="15" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A15" s="38"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="38"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="38"/>
-      <c r="G15" s="38"/>
-      <c r="H15" s="38"/>
-      <c r="I15" s="38"/>
-      <c r="J15" s="38"/>
       <c r="P15" s="9" t="s">
         <v>43</v>
       </c>
@@ -10722,17 +10607,7 @@
       </c>
     </row>
     <row r="16" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A16" s="38"/>
-      <c r="B16" s="38"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="38"/>
-      <c r="G16" s="38"/>
-      <c r="H16" s="38"/>
-      <c r="I16" s="38"/>
-      <c r="J16" s="38"/>
-      <c r="N16" s="29" t="s">
+      <c r="N16" s="43" t="s">
         <v>35</v>
       </c>
       <c r="O16" s="1" t="s">
@@ -10741,7 +10616,7 @@
       <c r="P16" s="12">
         <v>72.77</v>
       </c>
-      <c r="R16" s="29" t="s">
+      <c r="R16" s="43" t="s">
         <v>35</v>
       </c>
       <c r="S16" s="3" t="s">
@@ -10750,7 +10625,7 @@
       <c r="T16" s="14">
         <v>36.29</v>
       </c>
-      <c r="V16" s="29" t="s">
+      <c r="V16" s="43" t="s">
         <v>35</v>
       </c>
       <c r="W16" s="1" t="s">
@@ -10809,31 +10684,21 @@
       </c>
     </row>
     <row r="17" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A17" s="38"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="38"/>
-      <c r="G17" s="38"/>
-      <c r="H17" s="38"/>
-      <c r="I17" s="38"/>
-      <c r="J17" s="38"/>
-      <c r="N17" s="29"/>
+      <c r="N17" s="43"/>
       <c r="O17" s="3" t="s">
         <v>22</v>
       </c>
       <c r="P17" s="14">
         <v>48.86</v>
       </c>
-      <c r="R17" s="29"/>
+      <c r="R17" s="43"/>
       <c r="S17" s="3" t="s">
         <v>24</v>
       </c>
       <c r="T17" s="14">
         <v>77.44</v>
       </c>
-      <c r="V17" s="29"/>
+      <c r="V17" s="43"/>
       <c r="W17" s="3" t="s">
         <v>22</v>
       </c>
@@ -10890,17 +10755,7 @@
       </c>
     </row>
     <row r="18" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A18" s="38"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="38"/>
-      <c r="G18" s="38"/>
-      <c r="H18" s="38"/>
-      <c r="I18" s="38"/>
-      <c r="J18" s="38"/>
-      <c r="N18" s="29" t="s">
+      <c r="N18" s="43" t="s">
         <v>36</v>
       </c>
       <c r="O18" s="1" t="s">
@@ -10909,14 +10764,14 @@
       <c r="P18" s="12">
         <v>75.84</v>
       </c>
-      <c r="R18" s="29"/>
+      <c r="R18" s="43"/>
       <c r="S18" s="3" t="s">
         <v>25</v>
       </c>
       <c r="T18" s="14">
         <v>96.03</v>
       </c>
-      <c r="V18" s="29"/>
+      <c r="V18" s="43"/>
       <c r="W18" s="3" t="s">
         <v>23</v>
       </c>
@@ -10973,24 +10828,14 @@
       </c>
     </row>
     <row r="19" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A19" s="38"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="38"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="38"/>
-      <c r="I19" s="38"/>
-      <c r="J19" s="38"/>
-      <c r="N19" s="29"/>
+      <c r="N19" s="43"/>
       <c r="O19" s="3" t="s">
         <v>22</v>
       </c>
       <c r="P19" s="14">
         <v>64.19</v>
       </c>
-      <c r="R19" s="29" t="s">
+      <c r="R19" s="43" t="s">
         <v>36</v>
       </c>
       <c r="S19" s="3" t="s">
@@ -10999,7 +10844,7 @@
       <c r="T19" s="14">
         <v>56.54</v>
       </c>
-      <c r="V19" s="29" t="s">
+      <c r="V19" s="43" t="s">
         <v>36</v>
       </c>
       <c r="W19" s="1" t="s">
@@ -11016,17 +10861,7 @@
       </c>
     </row>
     <row r="20" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A20" s="38"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="38"/>
-      <c r="G20" s="38"/>
-      <c r="H20" s="38"/>
-      <c r="I20" s="38"/>
-      <c r="J20" s="38"/>
-      <c r="N20" s="29" t="s">
+      <c r="N20" s="43" t="s">
         <v>37</v>
       </c>
       <c r="O20" s="1" t="s">
@@ -11035,14 +10870,14 @@
       <c r="P20" s="12">
         <v>75.84</v>
       </c>
-      <c r="R20" s="29"/>
+      <c r="R20" s="43"/>
       <c r="S20" s="3" t="s">
         <v>24</v>
       </c>
       <c r="T20" s="14">
         <v>80.64</v>
       </c>
-      <c r="V20" s="29"/>
+      <c r="V20" s="43"/>
       <c r="W20" s="3" t="s">
         <v>22</v>
       </c>
@@ -11057,31 +10892,21 @@
       </c>
     </row>
     <row r="21" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A21" s="38"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="38"/>
-      <c r="H21" s="38"/>
-      <c r="I21" s="38"/>
-      <c r="J21" s="38"/>
-      <c r="N21" s="29"/>
+      <c r="N21" s="43"/>
       <c r="O21" s="3" t="s">
         <v>22</v>
       </c>
       <c r="P21" s="14">
         <v>63.19</v>
       </c>
-      <c r="R21" s="29"/>
+      <c r="R21" s="43"/>
       <c r="S21" s="3" t="s">
         <v>25</v>
       </c>
       <c r="T21" s="14">
         <v>121.95</v>
       </c>
-      <c r="V21" s="29"/>
+      <c r="V21" s="43"/>
       <c r="W21" s="3" t="s">
         <v>23</v>
       </c>
@@ -11096,17 +10921,7 @@
       </c>
     </row>
     <row r="22" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A22" s="38"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="38"/>
-      <c r="G22" s="38"/>
-      <c r="H22" s="38"/>
-      <c r="I22" s="38"/>
-      <c r="J22" s="38"/>
-      <c r="N22" s="29" t="s">
+      <c r="N22" s="43" t="s">
         <v>38</v>
       </c>
       <c r="O22" s="1" t="s">
@@ -11115,7 +10930,7 @@
       <c r="P22" s="12">
         <v>72.77</v>
       </c>
-      <c r="R22" s="29" t="s">
+      <c r="R22" s="43" t="s">
         <v>37</v>
       </c>
       <c r="S22" s="3" t="s">
@@ -11124,7 +10939,7 @@
       <c r="T22" s="14">
         <v>56.54</v>
       </c>
-      <c r="V22" s="29" t="s">
+      <c r="V22" s="43" t="s">
         <v>37</v>
       </c>
       <c r="W22" s="1" t="s">
@@ -11141,31 +10956,21 @@
       </c>
     </row>
     <row r="23" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A23" s="38"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="38"/>
-      <c r="G23" s="38"/>
-      <c r="H23" s="38"/>
-      <c r="I23" s="38"/>
-      <c r="J23" s="38"/>
-      <c r="N23" s="29"/>
+      <c r="N23" s="43"/>
       <c r="O23" s="3" t="s">
         <v>22</v>
       </c>
       <c r="P23" s="14">
         <v>48.86</v>
       </c>
-      <c r="R23" s="29"/>
+      <c r="R23" s="43"/>
       <c r="S23" s="3" t="s">
         <v>24</v>
       </c>
       <c r="T23" s="14">
         <v>82.53</v>
       </c>
-      <c r="V23" s="29"/>
+      <c r="V23" s="43"/>
       <c r="W23" s="3" t="s">
         <v>22</v>
       </c>
@@ -11180,7 +10985,7 @@
       </c>
     </row>
     <row r="24" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="N24" s="29" t="s">
+      <c r="N24" s="43" t="s">
         <v>39</v>
       </c>
       <c r="O24" s="1" t="s">
@@ -11189,14 +10994,14 @@
       <c r="P24" s="12">
         <v>76.03</v>
       </c>
-      <c r="R24" s="29"/>
+      <c r="R24" s="43"/>
       <c r="S24" s="3" t="s">
         <v>25</v>
       </c>
       <c r="T24" s="14">
         <v>162.11000000000001</v>
       </c>
-      <c r="V24" s="29"/>
+      <c r="V24" s="43"/>
       <c r="W24" s="3" t="s">
         <v>23</v>
       </c>
@@ -11211,14 +11016,14 @@
       </c>
     </row>
     <row r="25" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="N25" s="29"/>
+      <c r="N25" s="43"/>
       <c r="O25" s="3" t="s">
         <v>22</v>
       </c>
       <c r="P25" s="14">
         <v>120.51</v>
       </c>
-      <c r="R25" s="29" t="s">
+      <c r="R25" s="43" t="s">
         <v>38</v>
       </c>
       <c r="S25" s="3" t="s">
@@ -11227,7 +11032,7 @@
       <c r="T25" s="14">
         <v>36.130000000000003</v>
       </c>
-      <c r="V25" s="29" t="s">
+      <c r="V25" s="43" t="s">
         <v>38</v>
       </c>
       <c r="W25" s="1" t="s">
@@ -11244,20 +11049,20 @@
       </c>
     </row>
     <row r="26" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A26" s="31" t="s">
+      <c r="A26" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="B26" s="32"/>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="32"/>
-      <c r="I26" s="32"/>
-      <c r="J26" s="32"/>
-      <c r="K26" s="33"/>
-      <c r="N26" s="29" t="s">
+      <c r="B26" s="49"/>
+      <c r="C26" s="49"/>
+      <c r="D26" s="49"/>
+      <c r="E26" s="49"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="49"/>
+      <c r="H26" s="49"/>
+      <c r="I26" s="49"/>
+      <c r="J26" s="49"/>
+      <c r="K26" s="50"/>
+      <c r="N26" s="43" t="s">
         <v>40</v>
       </c>
       <c r="O26" s="1" t="s">
@@ -11266,14 +11071,14 @@
       <c r="P26" s="12">
         <v>67.260000000000005</v>
       </c>
-      <c r="R26" s="29"/>
+      <c r="R26" s="43"/>
       <c r="S26" s="3" t="s">
         <v>24</v>
       </c>
       <c r="T26" s="14">
         <v>77.44</v>
       </c>
-      <c r="V26" s="29"/>
+      <c r="V26" s="43"/>
       <c r="W26" s="3" t="s">
         <v>22</v>
       </c>
@@ -11317,21 +11122,21 @@
       <c r="K27" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="N27" s="29"/>
+      <c r="N27" s="43"/>
       <c r="O27" s="3" t="s">
         <v>22</v>
       </c>
       <c r="P27" s="14">
         <v>109.92</v>
       </c>
-      <c r="R27" s="29"/>
+      <c r="R27" s="43"/>
       <c r="S27" s="3" t="s">
         <v>25</v>
       </c>
       <c r="T27" s="14">
         <v>155.26</v>
       </c>
-      <c r="V27" s="29"/>
+      <c r="V27" s="43"/>
       <c r="W27" s="3" t="s">
         <v>23</v>
       </c>
@@ -11346,7 +11151,7 @@
       </c>
     </row>
     <row r="28" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A28" s="27" t="s">
+      <c r="A28" s="44" t="s">
         <v>9</v>
       </c>
       <c r="B28" s="1" t="s">
@@ -11357,15 +11162,15 @@
       <c r="E28" s="12">
         <v>72.77</v>
       </c>
-      <c r="F28" s="42"/>
-      <c r="G28" s="34"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="27"/>
       <c r="H28" s="12">
         <v>95.23</v>
       </c>
       <c r="I28" s="12"/>
       <c r="J28" s="13"/>
       <c r="K28" s="12"/>
-      <c r="N28" s="29" t="s">
+      <c r="N28" s="43" t="s">
         <v>41</v>
       </c>
       <c r="O28" s="1" t="s">
@@ -11374,7 +11179,7 @@
       <c r="P28" s="14">
         <v>66.27</v>
       </c>
-      <c r="R28" s="29" t="s">
+      <c r="R28" s="43" t="s">
         <v>39</v>
       </c>
       <c r="S28" s="3" t="s">
@@ -11383,7 +11188,7 @@
       <c r="T28" s="14">
         <v>103.04</v>
       </c>
-      <c r="V28" s="29" t="s">
+      <c r="V28" s="43" t="s">
         <v>39</v>
       </c>
       <c r="W28" s="1" t="s">
@@ -11400,7 +11205,7 @@
       </c>
     </row>
     <row r="29" spans="1:62" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="28"/>
+      <c r="A29" s="45"/>
       <c r="B29" s="3" t="s">
         <v>22</v>
       </c>
@@ -11413,31 +11218,31 @@
       <c r="E29" s="14">
         <v>48.86</v>
       </c>
-      <c r="F29" s="35">
+      <c r="F29" s="28">
         <v>36.29</v>
       </c>
-      <c r="G29" s="34"/>
+      <c r="G29" s="27"/>
       <c r="H29" s="14">
         <v>66.400000000000006</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="16"/>
       <c r="K29" s="14"/>
-      <c r="N29" s="29"/>
+      <c r="N29" s="43"/>
       <c r="O29" s="3" t="s">
         <v>22</v>
       </c>
       <c r="P29" s="14">
         <v>40.51</v>
       </c>
-      <c r="R29" s="29"/>
+      <c r="R29" s="43"/>
       <c r="S29" s="3" t="s">
         <v>24</v>
       </c>
       <c r="T29" s="14">
         <v>74.19</v>
       </c>
-      <c r="V29" s="29"/>
+      <c r="V29" s="43"/>
       <c r="W29" s="3" t="s">
         <v>22</v>
       </c>
@@ -11446,29 +11251,29 @@
       </c>
     </row>
     <row r="30" spans="1:62" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A30" s="28"/>
+      <c r="A30" s="45"/>
       <c r="B30" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C30" s="18"/>
       <c r="D30" s="20"/>
       <c r="E30" s="24"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="34"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="27"/>
       <c r="H30" s="14">
         <v>83.65</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="16"/>
       <c r="K30" s="14"/>
-      <c r="R30" s="29"/>
+      <c r="R30" s="43"/>
       <c r="S30" s="3" t="s">
         <v>25</v>
       </c>
       <c r="T30" s="14">
         <v>37.31</v>
       </c>
-      <c r="V30" s="29"/>
+      <c r="V30" s="43"/>
       <c r="W30" s="3" t="s">
         <v>23</v>
       </c>
@@ -11477,17 +11282,17 @@
       </c>
     </row>
     <row r="31" spans="1:62" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="28"/>
+      <c r="A31" s="45"/>
       <c r="B31" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C31" s="18"/>
       <c r="D31" s="20"/>
       <c r="E31" s="24"/>
-      <c r="F31" s="35">
+      <c r="F31" s="28">
         <v>77.44</v>
       </c>
-      <c r="G31" s="35">
+      <c r="G31" s="28">
         <v>155.71</v>
       </c>
       <c r="H31" s="20"/>
@@ -11496,7 +11301,7 @@
       </c>
       <c r="J31" s="16"/>
       <c r="K31" s="14"/>
-      <c r="R31" s="29" t="s">
+      <c r="R31" s="43" t="s">
         <v>40</v>
       </c>
       <c r="S31" s="3" t="s">
@@ -11505,7 +11310,7 @@
       <c r="T31" s="14">
         <v>81.790000000000006</v>
       </c>
-      <c r="V31" s="29" t="s">
+      <c r="V31" s="43" t="s">
         <v>40</v>
       </c>
       <c r="W31" s="1" t="s">
@@ -11516,31 +11321,31 @@
       </c>
     </row>
     <row r="32" spans="1:62" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A32" s="28"/>
+      <c r="A32" s="45"/>
       <c r="B32" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C32" s="18"/>
       <c r="D32" s="20"/>
       <c r="E32" s="24"/>
-      <c r="F32" s="44">
+      <c r="F32" s="35">
         <v>96.03</v>
       </c>
-      <c r="G32" s="35">
+      <c r="G32" s="28">
         <v>243.65</v>
       </c>
       <c r="H32" s="20"/>
       <c r="I32" s="14"/>
       <c r="J32" s="16"/>
       <c r="K32" s="14"/>
-      <c r="R32" s="29"/>
+      <c r="R32" s="43"/>
       <c r="S32" s="3" t="s">
         <v>24</v>
       </c>
       <c r="T32" s="14">
         <v>72.77</v>
       </c>
-      <c r="V32" s="29"/>
+      <c r="V32" s="43"/>
       <c r="W32" s="3" t="s">
         <v>22</v>
       </c>
@@ -11549,7 +11354,7 @@
       </c>
     </row>
     <row r="33" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A33" s="27" t="s">
+      <c r="A33" s="44" t="s">
         <v>10</v>
       </c>
       <c r="B33" s="1" t="s">
@@ -11560,22 +11365,22 @@
       <c r="E33" s="12">
         <v>75.84</v>
       </c>
-      <c r="F33" s="42"/>
+      <c r="F33" s="33"/>
       <c r="G33" s="17"/>
-      <c r="H33" s="41">
+      <c r="H33" s="32">
         <v>111.42</v>
       </c>
       <c r="I33" s="12"/>
       <c r="J33" s="13"/>
       <c r="K33" s="12"/>
-      <c r="R33" s="29"/>
+      <c r="R33" s="43"/>
       <c r="S33" s="3" t="s">
         <v>25</v>
       </c>
       <c r="T33" s="14">
         <v>28.61</v>
       </c>
-      <c r="V33" s="29"/>
+      <c r="V33" s="43"/>
       <c r="W33" s="3" t="s">
         <v>23</v>
       </c>
@@ -11590,7 +11395,7 @@
       </c>
     </row>
     <row r="34" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A34" s="28"/>
+      <c r="A34" s="45"/>
       <c r="B34" s="3" t="s">
         <v>22</v>
       </c>
@@ -11603,11 +11408,11 @@
       <c r="E34" s="14">
         <v>64.19</v>
       </c>
-      <c r="F34" s="35">
+      <c r="F34" s="28">
         <v>56.54</v>
       </c>
       <c r="G34" s="24"/>
-      <c r="H34" s="35">
+      <c r="H34" s="28">
         <v>94.18</v>
       </c>
       <c r="I34" s="14"/>
@@ -11616,7 +11421,7 @@
       <c r="P34" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="R34" s="29" t="s">
+      <c r="R34" s="43" t="s">
         <v>41</v>
       </c>
       <c r="S34" s="3" t="s">
@@ -11625,7 +11430,7 @@
       <c r="T34" s="14">
         <v>36.32</v>
       </c>
-      <c r="V34" s="29" t="s">
+      <c r="V34" s="43" t="s">
         <v>41</v>
       </c>
       <c r="W34" s="1" t="s">
@@ -11642,22 +11447,22 @@
       </c>
     </row>
     <row r="35" spans="1:62" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A35" s="28"/>
+      <c r="A35" s="45"/>
       <c r="B35" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C35" s="18"/>
       <c r="D35" s="20"/>
       <c r="E35" s="24"/>
-      <c r="F35" s="43"/>
+      <c r="F35" s="34"/>
       <c r="G35" s="24"/>
-      <c r="H35" s="35">
+      <c r="H35" s="28">
         <v>116.22</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="16"/>
       <c r="K35" s="14"/>
-      <c r="N35" s="29" t="s">
+      <c r="N35" s="43" t="s">
         <v>35</v>
       </c>
       <c r="O35" s="3" t="s">
@@ -11666,14 +11471,14 @@
       <c r="P35" s="14">
         <v>155.71</v>
       </c>
-      <c r="R35" s="29"/>
+      <c r="R35" s="43"/>
       <c r="S35" s="3" t="s">
         <v>24</v>
       </c>
       <c r="T35" s="14">
         <v>74.75</v>
       </c>
-      <c r="V35" s="29"/>
+      <c r="V35" s="43"/>
       <c r="W35" s="3" t="s">
         <v>22</v>
       </c>
@@ -11688,40 +11493,40 @@
       </c>
     </row>
     <row r="36" spans="1:62" x14ac:dyDescent="0.45">
-      <c r="A36" s="28"/>
+      <c r="A36" s="45"/>
       <c r="B36" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C36" s="18"/>
       <c r="D36" s="20"/>
       <c r="E36" s="24"/>
-      <c r="F36" s="35">
+      <c r="F36" s="28">
         <v>80.64</v>
       </c>
       <c r="G36" s="14">
         <v>120.93</v>
       </c>
-      <c r="H36" s="34"/>
+      <c r="H36" s="27"/>
       <c r="I36" s="14">
         <v>56.32</v>
       </c>
       <c r="J36" s="16"/>
       <c r="K36" s="14"/>
-      <c r="N36" s="29"/>
+      <c r="N36" s="43"/>
       <c r="O36" s="3" t="s">
         <v>25</v>
       </c>
       <c r="P36" s="14">
         <v>243.65</v>
       </c>
-      <c r="R36" s="29"/>
+      <c r="R36" s="43"/>
       <c r="S36" s="3" t="s">
         <v>25</v>
       </c>
       <c r="T36" s="14">
         <v>93.73</v>
       </c>
-      <c r="V36" s="29"/>
+      <c r="V36" s="43"/>
       <c r="W36" s="3" t="s">
         <v>23</v>
       </c>
@@ -11736,24 +11541,24 @@
       </c>
     </row>
     <row r="37" spans="1:62" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A37" s="28"/>
+      <c r="A37" s="45"/>
       <c r="B37" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C37" s="18"/>
       <c r="D37" s="20"/>
       <c r="E37" s="24"/>
-      <c r="F37" s="44">
+      <c r="F37" s="35">
         <v>121.95</v>
       </c>
-      <c r="G37" s="45">
+      <c r="G37" s="36">
         <v>272.77</v>
       </c>
-      <c r="H37" s="34"/>
+      <c r="H37" s="27"/>
       <c r="I37" s="14"/>
       <c r="J37" s="16"/>
       <c r="K37" s="14"/>
-      <c r="N37" s="29" t="s">
+      <c r="N37" s="43" t="s">
         <v>36</v>
       </c>
       <c r="O37" s="3" t="s">
@@ -11764,7 +11569,7 @@
       </c>
     </row>
     <row r="38" spans="1:62" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A38" s="28" t="s">
+      <c r="A38" s="45" t="s">
         <v>11</v>
       </c>
       <c r="B38" s="1" t="s">
@@ -11775,7 +11580,7 @@
       <c r="E38" s="12">
         <v>75.84</v>
       </c>
-      <c r="F38" s="42"/>
+      <c r="F38" s="33"/>
       <c r="G38" s="17"/>
       <c r="H38" s="12">
         <v>111.42</v>
@@ -11783,7 +11588,7 @@
       <c r="I38" s="12"/>
       <c r="J38" s="13"/>
       <c r="K38" s="12"/>
-      <c r="N38" s="29"/>
+      <c r="N38" s="43"/>
       <c r="O38" s="3" t="s">
         <v>25</v>
       </c>
@@ -11792,7 +11597,7 @@
       </c>
     </row>
     <row r="39" spans="1:62" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A39" s="28"/>
+      <c r="A39" s="45"/>
       <c r="B39" s="3" t="s">
         <v>22</v>
       </c>
@@ -11815,7 +11620,7 @@
       <c r="I39" s="14"/>
       <c r="J39" s="16"/>
       <c r="K39" s="14"/>
-      <c r="N39" s="29" t="s">
+      <c r="N39" s="43" t="s">
         <v>37</v>
       </c>
       <c r="O39" s="3" t="s">
@@ -11826,7 +11631,7 @@
       </c>
     </row>
     <row r="40" spans="1:62" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A40" s="28"/>
+      <c r="A40" s="45"/>
       <c r="B40" s="3" t="s">
         <v>23</v>
       </c>
@@ -11841,7 +11646,7 @@
       <c r="I40" s="14"/>
       <c r="J40" s="16"/>
       <c r="K40" s="14"/>
-      <c r="N40" s="29"/>
+      <c r="N40" s="43"/>
       <c r="O40" s="3" t="s">
         <v>25</v>
       </c>
@@ -11853,7 +11658,7 @@
       </c>
     </row>
     <row r="41" spans="1:62" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A41" s="28"/>
+      <c r="A41" s="45"/>
       <c r="B41" s="3" t="s">
         <v>24</v>
       </c>
@@ -11872,7 +11677,7 @@
       </c>
       <c r="J41" s="16"/>
       <c r="K41" s="14"/>
-      <c r="N41" s="29" t="s">
+      <c r="N41" s="43" t="s">
         <v>38</v>
       </c>
       <c r="O41" s="3" t="s">
@@ -11889,24 +11694,24 @@
       </c>
     </row>
     <row r="42" spans="1:62" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A42" s="28"/>
+      <c r="A42" s="45"/>
       <c r="B42" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C42" s="18"/>
       <c r="D42" s="20"/>
       <c r="E42" s="20"/>
-      <c r="F42" s="45">
+      <c r="F42" s="36">
         <v>162.11000000000001</v>
       </c>
-      <c r="G42" s="45">
+      <c r="G42" s="36">
         <v>301.92</v>
       </c>
       <c r="H42" s="20"/>
       <c r="I42" s="14"/>
       <c r="J42" s="16"/>
       <c r="K42" s="14"/>
-      <c r="N42" s="29"/>
+      <c r="N42" s="43"/>
       <c r="O42" s="3" t="s">
         <v>25</v>
       </c>
@@ -11921,7 +11726,7 @@
       </c>
     </row>
     <row r="43" spans="1:62" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A43" s="27" t="s">
+      <c r="A43" s="44" t="s">
         <v>12</v>
       </c>
       <c r="B43" s="1" t="s">
@@ -11940,7 +11745,7 @@
       <c r="I43" s="12"/>
       <c r="J43" s="13"/>
       <c r="K43" s="12"/>
-      <c r="N43" s="29" t="s">
+      <c r="N43" s="43" t="s">
         <v>39</v>
       </c>
       <c r="O43" s="3" t="s">
@@ -11957,7 +11762,7 @@
       </c>
     </row>
     <row r="44" spans="1:62" x14ac:dyDescent="0.45">
-      <c r="A44" s="28"/>
+      <c r="A44" s="45"/>
       <c r="B44" s="3" t="s">
         <v>22</v>
       </c>
@@ -11980,7 +11785,7 @@
       <c r="I44" s="14"/>
       <c r="J44" s="16"/>
       <c r="K44" s="14"/>
-      <c r="N44" s="29"/>
+      <c r="N44" s="43"/>
       <c r="O44" s="3" t="s">
         <v>25</v>
       </c>
@@ -11995,7 +11800,7 @@
       </c>
     </row>
     <row r="45" spans="1:62" x14ac:dyDescent="0.45">
-      <c r="A45" s="28"/>
+      <c r="A45" s="45"/>
       <c r="B45" s="3" t="s">
         <v>23</v>
       </c>
@@ -12010,7 +11815,7 @@
       <c r="I45" s="14"/>
       <c r="J45" s="16"/>
       <c r="K45" s="14"/>
-      <c r="N45" s="29" t="s">
+      <c r="N45" s="43" t="s">
         <v>40</v>
       </c>
       <c r="O45" s="3" t="s">
@@ -12027,7 +11832,7 @@
       </c>
     </row>
     <row r="46" spans="1:62" x14ac:dyDescent="0.45">
-      <c r="A46" s="28"/>
+      <c r="A46" s="45"/>
       <c r="B46" s="3" t="s">
         <v>24</v>
       </c>
@@ -12046,7 +11851,7 @@
       </c>
       <c r="J46" s="16"/>
       <c r="K46" s="14"/>
-      <c r="N46" s="29"/>
+      <c r="N46" s="43"/>
       <c r="O46" s="3" t="s">
         <v>25</v>
       </c>
@@ -12061,24 +11866,24 @@
       </c>
     </row>
     <row r="47" spans="1:62" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A47" s="28"/>
+      <c r="A47" s="45"/>
       <c r="B47" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C47" s="18"/>
       <c r="D47" s="20"/>
       <c r="E47" s="20"/>
-      <c r="F47" s="45">
+      <c r="F47" s="36">
         <v>155.26</v>
       </c>
-      <c r="G47" s="45">
+      <c r="G47" s="36">
         <v>282.66000000000003</v>
       </c>
       <c r="H47" s="20"/>
       <c r="I47" s="14"/>
       <c r="J47" s="16"/>
       <c r="K47" s="14"/>
-      <c r="N47" s="29" t="s">
+      <c r="N47" s="43" t="s">
         <v>41</v>
       </c>
       <c r="O47" s="3" t="s">
@@ -12095,7 +11900,7 @@
       </c>
     </row>
     <row r="48" spans="1:62" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A48" s="27" t="s">
+      <c r="A48" s="44" t="s">
         <v>13</v>
       </c>
       <c r="B48" s="1" t="s">
@@ -12114,7 +11919,7 @@
       <c r="I48" s="12"/>
       <c r="J48" s="13"/>
       <c r="K48" s="12"/>
-      <c r="N48" s="29"/>
+      <c r="N48" s="43"/>
       <c r="O48" s="3" t="s">
         <v>25</v>
       </c>
@@ -12122,8 +11927,8 @@
         <v>238.53</v>
       </c>
     </row>
-    <row r="49" spans="1:25" x14ac:dyDescent="0.45">
-      <c r="A49" s="28"/>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A49" s="45"/>
       <c r="B49" s="3" t="s">
         <v>22</v>
       </c>
@@ -12147,8 +11952,8 @@
       <c r="J49" s="16"/>
       <c r="K49" s="14"/>
     </row>
-    <row r="50" spans="1:25" x14ac:dyDescent="0.45">
-      <c r="A50" s="28"/>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A50" s="45"/>
       <c r="B50" s="3" t="s">
         <v>23</v>
       </c>
@@ -12163,20 +11968,9 @@
       <c r="I50" s="14"/>
       <c r="J50" s="16"/>
       <c r="K50" s="14"/>
-      <c r="O50" s="38"/>
-      <c r="P50" s="38"/>
-      <c r="Q50" s="38"/>
-      <c r="R50" s="38"/>
-      <c r="S50" s="38"/>
-      <c r="T50" s="38"/>
-      <c r="U50" s="38"/>
-      <c r="V50" s="38"/>
-      <c r="W50" s="38"/>
-      <c r="X50" s="38"/>
-      <c r="Y50" s="38"/>
     </row>
-    <row r="51" spans="1:25" x14ac:dyDescent="0.45">
-      <c r="A51" s="28"/>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A51" s="45"/>
       <c r="B51" s="3" t="s">
         <v>24</v>
       </c>
@@ -12196,18 +11990,18 @@
       <c r="J51" s="16"/>
       <c r="K51" s="14"/>
     </row>
-    <row r="52" spans="1:25" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A52" s="28"/>
+    <row r="52" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A52" s="45"/>
       <c r="B52" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C52" s="18"/>
       <c r="D52" s="20"/>
       <c r="E52" s="20"/>
-      <c r="F52" s="45">
+      <c r="F52" s="36">
         <v>37.31</v>
       </c>
-      <c r="G52" s="45">
+      <c r="G52" s="36">
         <v>215.42</v>
       </c>
       <c r="H52" s="20"/>
@@ -12215,8 +12009,8 @@
       <c r="J52" s="16"/>
       <c r="K52" s="14"/>
     </row>
-    <row r="53" spans="1:25" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A53" s="27" t="s">
+    <row r="53" spans="1:13" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A53" s="44" t="s">
         <v>14</v>
       </c>
       <c r="B53" s="1" t="s">
@@ -12236,8 +12030,8 @@
       <c r="J53" s="13"/>
       <c r="K53" s="12"/>
     </row>
-    <row r="54" spans="1:25" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A54" s="28"/>
+    <row r="54" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A54" s="45"/>
       <c r="B54" s="3" t="s">
         <v>22</v>
       </c>
@@ -12261,8 +12055,8 @@
       <c r="J54" s="16"/>
       <c r="K54" s="14"/>
     </row>
-    <row r="55" spans="1:25" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A55" s="28"/>
+    <row r="55" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A55" s="45"/>
       <c r="B55" s="3" t="s">
         <v>23</v>
       </c>
@@ -12277,10 +12071,10 @@
       <c r="I55" s="14"/>
       <c r="J55" s="16"/>
       <c r="K55" s="14"/>
-      <c r="M55" s="40"/>
+      <c r="M55" s="31"/>
     </row>
-    <row r="56" spans="1:25" x14ac:dyDescent="0.45">
-      <c r="A56" s="28"/>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A56" s="45"/>
       <c r="B56" s="3" t="s">
         <v>24</v>
       </c>
@@ -12300,27 +12094,27 @@
       <c r="J56" s="16"/>
       <c r="K56" s="14"/>
     </row>
-    <row r="57" spans="1:25" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A57" s="28"/>
+    <row r="57" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A57" s="45"/>
       <c r="B57" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C57" s="18"/>
       <c r="D57" s="20"/>
-      <c r="E57" s="46"/>
-      <c r="F57" s="45">
+      <c r="E57" s="37"/>
+      <c r="F57" s="36">
         <v>28.61</v>
       </c>
-      <c r="G57" s="45">
+      <c r="G57" s="36">
         <v>198.66</v>
       </c>
-      <c r="H57" s="46"/>
-      <c r="I57" s="45"/>
+      <c r="H57" s="37"/>
+      <c r="I57" s="36"/>
       <c r="J57" s="16"/>
       <c r="K57" s="14"/>
     </row>
-    <row r="58" spans="1:25" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A58" s="27" t="s">
+    <row r="58" spans="1:13" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A58" s="44" t="s">
         <v>15</v>
       </c>
       <c r="B58" s="1" t="s">
@@ -12340,8 +12134,8 @@
       <c r="J58" s="16"/>
       <c r="K58" s="14"/>
     </row>
-    <row r="59" spans="1:25" x14ac:dyDescent="0.45">
-      <c r="A59" s="28"/>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A59" s="45"/>
       <c r="B59" s="3" t="s">
         <v>22</v>
       </c>
@@ -12365,8 +12159,8 @@
       <c r="J59" s="16"/>
       <c r="K59" s="14"/>
     </row>
-    <row r="60" spans="1:25" x14ac:dyDescent="0.45">
-      <c r="A60" s="28"/>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A60" s="45"/>
       <c r="B60" s="3" t="s">
         <v>23</v>
       </c>
@@ -12382,8 +12176,8 @@
       <c r="J60" s="16"/>
       <c r="K60" s="14"/>
     </row>
-    <row r="61" spans="1:25" x14ac:dyDescent="0.45">
-      <c r="A61" s="28"/>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A61" s="45"/>
       <c r="B61" s="3" t="s">
         <v>24</v>
       </c>
@@ -12403,33 +12197,33 @@
       <c r="J61" s="16"/>
       <c r="K61" s="14"/>
     </row>
-    <row r="62" spans="1:25" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A62" s="28"/>
+    <row r="62" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A62" s="45"/>
       <c r="B62" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C62" s="18"/>
-      <c r="D62" s="46"/>
-      <c r="E62" s="47"/>
-      <c r="F62" s="45">
+      <c r="D62" s="37"/>
+      <c r="E62" s="38"/>
+      <c r="F62" s="36">
         <v>93.73</v>
       </c>
-      <c r="G62" s="45">
+      <c r="G62" s="36">
         <v>238.53</v>
       </c>
-      <c r="H62" s="46"/>
-      <c r="I62" s="45"/>
+      <c r="H62" s="37"/>
+      <c r="I62" s="36"/>
       <c r="J62" s="16"/>
       <c r="K62" s="14"/>
     </row>
-    <row r="63" spans="1:25" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A63" s="27" t="s">
+    <row r="63" spans="1:13" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A63" s="44" t="s">
         <v>67</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C63" s="49"/>
+      <c r="C63" s="40"/>
       <c r="D63" s="20"/>
       <c r="E63" s="14">
         <v>67.010000000000005</v>
@@ -12443,8 +12237,8 @@
       <c r="J63" s="12"/>
       <c r="K63" s="12"/>
     </row>
-    <row r="64" spans="1:25" x14ac:dyDescent="0.45">
-      <c r="A64" s="28"/>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A64" s="45"/>
       <c r="B64" s="3" t="s">
         <v>22</v>
       </c>
@@ -12452,25 +12246,25 @@
         <v>23.26</v>
       </c>
       <c r="D64" s="15">
-        <v>45.54</v>
+        <v>45.6</v>
       </c>
       <c r="E64" s="14">
-        <v>101.44</v>
-      </c>
-      <c r="F64" s="36"/>
+        <v>101.7</v>
+      </c>
+      <c r="F64" s="29">
+        <v>88.13</v>
+      </c>
       <c r="G64" s="20"/>
-      <c r="H64" s="36">
-        <v>123.71</v>
-      </c>
+      <c r="H64" s="29"/>
       <c r="I64" s="14"/>
       <c r="J64" s="15"/>
       <c r="K64" s="14"/>
-      <c r="M64" s="39" t="s">
+      <c r="M64" s="30" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="65" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A65" s="28"/>
+      <c r="A65" s="45"/>
       <c r="B65" s="3" t="s">
         <v>23</v>
       </c>
@@ -12479,64 +12273,70 @@
       <c r="E65" s="20"/>
       <c r="F65" s="24"/>
       <c r="G65" s="20"/>
-      <c r="H65" s="36"/>
+      <c r="H65" s="29"/>
       <c r="I65" s="14"/>
       <c r="J65" s="15"/>
       <c r="K65" s="14"/>
     </row>
     <row r="66" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A66" s="28"/>
+      <c r="A66" s="45"/>
       <c r="B66" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C66" s="26"/>
       <c r="D66" s="20"/>
       <c r="E66" s="20"/>
-      <c r="F66" s="36"/>
-      <c r="G66" s="36"/>
+      <c r="F66" s="29">
+        <v>74.819999999999993</v>
+      </c>
+      <c r="G66" s="29">
+        <v>115.68</v>
+      </c>
       <c r="H66" s="20"/>
       <c r="I66" s="14">
-        <v>54.58</v>
+        <v>53.41</v>
       </c>
       <c r="J66" s="15"/>
       <c r="K66" s="14"/>
     </row>
     <row r="67" spans="1:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A67" s="30"/>
+      <c r="A67" s="46"/>
       <c r="B67" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C67" s="50"/>
-      <c r="D67" s="46"/>
-      <c r="E67" s="46"/>
-      <c r="F67" s="45">
+      <c r="C67" s="41"/>
+      <c r="D67" s="37"/>
+      <c r="E67" s="37"/>
+      <c r="F67" s="36">
         <v>24.67</v>
       </c>
-      <c r="G67" s="51"/>
-      <c r="H67" s="46"/>
-      <c r="I67" s="45"/>
-      <c r="J67" s="48"/>
-      <c r="K67" s="45"/>
+      <c r="G67" s="42">
+        <v>202.98</v>
+      </c>
+      <c r="H67" s="37"/>
+      <c r="I67" s="36"/>
+      <c r="J67" s="39"/>
+      <c r="K67" s="36"/>
     </row>
     <row r="68" spans="1:20" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
     <row r="69" spans="1:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="70" spans="1:20" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A70" s="31" t="s">
+      <c r="A70" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="B70" s="32"/>
-      <c r="C70" s="32"/>
-      <c r="D70" s="32"/>
-      <c r="E70" s="32"/>
-      <c r="F70" s="32"/>
-      <c r="G70" s="32"/>
-      <c r="H70" s="32"/>
-      <c r="I70" s="32"/>
-      <c r="J70" s="32"/>
-      <c r="K70" s="32"/>
-      <c r="L70" s="32"/>
-      <c r="M70" s="32"/>
-      <c r="N70" s="33"/>
+      <c r="B70" s="49"/>
+      <c r="C70" s="49"/>
+      <c r="D70" s="49"/>
+      <c r="E70" s="49"/>
+      <c r="F70" s="49"/>
+      <c r="G70" s="49"/>
+      <c r="H70" s="49"/>
+      <c r="I70" s="49"/>
+      <c r="J70" s="49"/>
+      <c r="K70" s="49"/>
+      <c r="L70" s="49"/>
+      <c r="M70" s="49"/>
+      <c r="N70" s="50"/>
     </row>
     <row r="71" spans="1:20" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A71" s="8"/>
@@ -12585,7 +12385,7 @@
       </c>
     </row>
     <row r="72" spans="1:20" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A72" s="27" t="s">
+      <c r="A72" s="44" t="s">
         <v>9</v>
       </c>
       <c r="B72" s="1" t="s">
@@ -12629,7 +12429,7 @@
       <c r="T72" s="2"/>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A73" s="28"/>
+      <c r="A73" s="45"/>
       <c r="B73" s="3" t="s">
         <v>19</v>
       </c>
@@ -12679,7 +12479,7 @@
       </c>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A74" s="28"/>
+      <c r="A74" s="45"/>
       <c r="B74" s="3" t="s">
         <v>20</v>
       </c>
@@ -12720,7 +12520,7 @@
       <c r="S74" s="7"/>
     </row>
     <row r="75" spans="1:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A75" s="30"/>
+      <c r="A75" s="46"/>
       <c r="B75" s="4" t="s">
         <v>26</v>
       </c>
@@ -12762,7 +12562,7 @@
       <c r="T75" s="5"/>
     </row>
     <row r="76" spans="1:20" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A76" s="27" t="s">
+      <c r="A76" s="44" t="s">
         <v>10</v>
       </c>
       <c r="B76" s="1" t="s">
@@ -12806,7 +12606,7 @@
       <c r="T76" s="2"/>
     </row>
     <row r="77" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A77" s="28"/>
+      <c r="A77" s="45"/>
       <c r="B77" s="3" t="s">
         <v>19</v>
       </c>
@@ -12847,7 +12647,7 @@
       <c r="S77" s="7"/>
     </row>
     <row r="78" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A78" s="28"/>
+      <c r="A78" s="45"/>
       <c r="B78" s="3" t="s">
         <v>20</v>
       </c>
@@ -12888,7 +12688,7 @@
       <c r="S78" s="7"/>
     </row>
     <row r="79" spans="1:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A79" s="30"/>
+      <c r="A79" s="46"/>
       <c r="B79" s="4" t="s">
         <v>26</v>
       </c>
@@ -12930,7 +12730,7 @@
       <c r="T79" s="5"/>
     </row>
     <row r="80" spans="1:20" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A80" s="28" t="s">
+      <c r="A80" s="45" t="s">
         <v>11</v>
       </c>
       <c r="B80" s="1" t="s">
@@ -12974,7 +12774,7 @@
       <c r="T80" s="2"/>
     </row>
     <row r="81" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A81" s="28"/>
+      <c r="A81" s="45"/>
       <c r="B81" s="3" t="s">
         <v>19</v>
       </c>
@@ -13015,7 +12815,7 @@
       <c r="S81" s="7"/>
     </row>
     <row r="82" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A82" s="28"/>
+      <c r="A82" s="45"/>
       <c r="B82" s="3" t="s">
         <v>20</v>
       </c>
@@ -13056,7 +12856,7 @@
       <c r="S82" s="7"/>
     </row>
     <row r="83" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A83" s="28"/>
+      <c r="A83" s="45"/>
       <c r="B83" s="3" t="s">
         <v>29</v>
       </c>
@@ -13097,7 +12897,7 @@
       <c r="S83" s="7"/>
     </row>
     <row r="84" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A84" s="28"/>
+      <c r="A84" s="45"/>
       <c r="B84" s="3" t="s">
         <v>30</v>
       </c>
@@ -13138,7 +12938,7 @@
       <c r="S84" s="7"/>
     </row>
     <row r="85" spans="1:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A85" s="30"/>
+      <c r="A85" s="46"/>
       <c r="B85" s="4" t="s">
         <v>26</v>
       </c>
@@ -13180,7 +12980,7 @@
       <c r="T85" s="5"/>
     </row>
     <row r="86" spans="1:20" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A86" s="27" t="s">
+      <c r="A86" s="44" t="s">
         <v>12</v>
       </c>
       <c r="B86" s="1" t="s">
@@ -13224,7 +13024,7 @@
       <c r="T86" s="2"/>
     </row>
     <row r="87" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A87" s="28"/>
+      <c r="A87" s="45"/>
       <c r="B87" s="3" t="s">
         <v>19</v>
       </c>
@@ -13274,7 +13074,7 @@
       </c>
     </row>
     <row r="88" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A88" s="28"/>
+      <c r="A88" s="45"/>
       <c r="B88" s="3" t="s">
         <v>20</v>
       </c>
@@ -13315,7 +13115,7 @@
       <c r="S88" s="7"/>
     </row>
     <row r="89" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A89" s="28"/>
+      <c r="A89" s="45"/>
       <c r="B89" s="3" t="s">
         <v>29</v>
       </c>
@@ -13356,7 +13156,7 @@
       <c r="S89" s="7"/>
     </row>
     <row r="90" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A90" s="28"/>
+      <c r="A90" s="45"/>
       <c r="B90" s="3" t="s">
         <v>30</v>
       </c>
@@ -13397,7 +13197,7 @@
       <c r="S90" s="7"/>
     </row>
     <row r="91" spans="1:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A91" s="30"/>
+      <c r="A91" s="46"/>
       <c r="B91" s="4" t="s">
         <v>26</v>
       </c>
@@ -13439,7 +13239,7 @@
       <c r="T91" s="5"/>
     </row>
     <row r="92" spans="1:20" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A92" s="27" t="s">
+      <c r="A92" s="44" t="s">
         <v>13</v>
       </c>
       <c r="B92" s="1" t="s">
@@ -13483,7 +13283,7 @@
       <c r="T92" s="2"/>
     </row>
     <row r="93" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A93" s="28"/>
+      <c r="A93" s="45"/>
       <c r="B93" s="3" t="s">
         <v>19</v>
       </c>
@@ -13524,7 +13324,7 @@
       <c r="S93" s="7"/>
     </row>
     <row r="94" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A94" s="28"/>
+      <c r="A94" s="45"/>
       <c r="B94" s="3" t="s">
         <v>20</v>
       </c>
@@ -13565,7 +13365,7 @@
       <c r="S94" s="7"/>
     </row>
     <row r="95" spans="1:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A95" s="30"/>
+      <c r="A95" s="46"/>
       <c r="B95" s="4" t="s">
         <v>26</v>
       </c>
@@ -13607,7 +13407,7 @@
       <c r="T95" s="5"/>
     </row>
     <row r="96" spans="1:20" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A96" s="27" t="s">
+      <c r="A96" s="44" t="s">
         <v>14</v>
       </c>
       <c r="B96" s="1" t="s">
@@ -13651,7 +13451,7 @@
       <c r="T96" s="2"/>
     </row>
     <row r="97" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A97" s="28"/>
+      <c r="A97" s="45"/>
       <c r="B97" s="3" t="s">
         <v>19</v>
       </c>
@@ -13701,7 +13501,7 @@
       </c>
     </row>
     <row r="98" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A98" s="28"/>
+      <c r="A98" s="45"/>
       <c r="B98" s="3" t="s">
         <v>20</v>
       </c>
@@ -13742,7 +13542,7 @@
       <c r="S98" s="7"/>
     </row>
     <row r="99" spans="1:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A99" s="30"/>
+      <c r="A99" s="46"/>
       <c r="B99" s="4" t="s">
         <v>26</v>
       </c>
@@ -13784,7 +13584,7 @@
       <c r="T99" s="5"/>
     </row>
     <row r="100" spans="1:20" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A100" s="27" t="s">
+      <c r="A100" s="44" t="s">
         <v>15</v>
       </c>
       <c r="B100" s="1" t="s">
@@ -13827,7 +13627,7 @@
       <c r="S100" s="7"/>
     </row>
     <row r="101" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A101" s="28"/>
+      <c r="A101" s="45"/>
       <c r="B101" s="3" t="s">
         <v>19</v>
       </c>
@@ -13868,7 +13668,7 @@
       <c r="S101" s="7"/>
     </row>
     <row r="102" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A102" s="28"/>
+      <c r="A102" s="45"/>
       <c r="B102" s="3" t="s">
         <v>20</v>
       </c>
@@ -13909,7 +13709,7 @@
       <c r="S102" s="7"/>
     </row>
     <row r="103" spans="1:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A103" s="30"/>
+      <c r="A103" s="46"/>
       <c r="B103" s="4" t="s">
         <v>26</v>
       </c>
@@ -13953,20 +13753,11 @@
     <row r="104" spans="1:20" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A43:A47"/>
-    <mergeCell ref="N43:N44"/>
-    <mergeCell ref="N45:N46"/>
-    <mergeCell ref="N22:N23"/>
-    <mergeCell ref="N24:N25"/>
-    <mergeCell ref="N26:N27"/>
-    <mergeCell ref="N28:N29"/>
-    <mergeCell ref="N41:N42"/>
-    <mergeCell ref="N20:N21"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A28:A32"/>
     <mergeCell ref="A33:A37"/>
     <mergeCell ref="A38:A42"/>
-    <mergeCell ref="A92:A95"/>
+    <mergeCell ref="A43:A47"/>
     <mergeCell ref="A96:A99"/>
     <mergeCell ref="A100:A103"/>
     <mergeCell ref="A13:G13"/>
@@ -13981,25 +13772,34 @@
     <mergeCell ref="A70:N70"/>
     <mergeCell ref="N16:N17"/>
     <mergeCell ref="N18:N19"/>
-    <mergeCell ref="R22:R24"/>
-    <mergeCell ref="R25:R27"/>
-    <mergeCell ref="R28:R30"/>
+    <mergeCell ref="N20:N21"/>
+    <mergeCell ref="N43:N44"/>
     <mergeCell ref="A63:A67"/>
     <mergeCell ref="N47:N48"/>
+    <mergeCell ref="N37:N38"/>
+    <mergeCell ref="N39:N40"/>
+    <mergeCell ref="A92:A95"/>
+    <mergeCell ref="N45:N46"/>
+    <mergeCell ref="N41:N42"/>
+    <mergeCell ref="N35:N36"/>
     <mergeCell ref="V16:V18"/>
     <mergeCell ref="V19:V21"/>
     <mergeCell ref="V22:V24"/>
     <mergeCell ref="V25:V27"/>
     <mergeCell ref="V28:V30"/>
+    <mergeCell ref="R22:R24"/>
+    <mergeCell ref="R25:R27"/>
+    <mergeCell ref="R28:R30"/>
+    <mergeCell ref="N22:N23"/>
+    <mergeCell ref="N24:N25"/>
+    <mergeCell ref="N26:N27"/>
+    <mergeCell ref="N28:N29"/>
+    <mergeCell ref="R16:R18"/>
+    <mergeCell ref="R19:R21"/>
     <mergeCell ref="V31:V33"/>
     <mergeCell ref="V34:V36"/>
     <mergeCell ref="R31:R33"/>
     <mergeCell ref="R34:R36"/>
-    <mergeCell ref="N35:N36"/>
-    <mergeCell ref="N37:N38"/>
-    <mergeCell ref="N39:N40"/>
-    <mergeCell ref="R16:R18"/>
-    <mergeCell ref="R19:R21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>